<commit_message>
setting up to work on carks
</commit_message>
<xml_diff>
--- a/artifacts/input.xlsx
+++ b/artifacts/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E505E6-3949-47CA-9669-ABB11F946ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F9537B-57AA-43CD-886E-58E3AA2E1E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>Field Name</t>
   </si>
@@ -216,6 +216,18 @@
   </si>
   <si>
     <t>PM FY2031</t>
+  </si>
+  <si>
+    <t>No. of 4 wheelers</t>
+  </si>
+  <si>
+    <t>Rate per 4 wheeler</t>
+  </si>
+  <si>
+    <t>No. of 2 wheelers</t>
+  </si>
+  <si>
+    <t>Rate per 2 wheeler</t>
   </si>
 </sst>
 </file>
@@ -326,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -346,6 +358,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -680,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79635125-D570-4C1E-9257-DC9C160143A9}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" bestFit="1" customWidth="1"/>
@@ -944,7 +958,7 @@
         <v>7.1099999999999997E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="13" t="s">
         <v>43</v>
       </c>
@@ -952,131 +966,163 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="13" t="s">
+    <row r="35" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="15">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="15">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="15">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B35">
+      <c r="B39">
         <v>110.5</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" s="13" t="s">
+    <row r="40" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B36">
+      <c r="B40">
         <v>2500000</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" s="13" t="s">
+    <row r="41" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B37">
+      <c r="B41">
         <v>14000000</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" s="13" t="s">
+    <row r="42" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="13" t="s">
         <v>47</v>
-      </c>
-      <c r="B38">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39">
-        <v>15000000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40">
-        <v>14000000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B41">
-        <v>12000000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" s="13" t="s">
-        <v>51</v>
       </c>
       <c r="B42">
         <v>5000000</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43">
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44">
+        <v>14000000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B43">
+      <c r="B47">
         <v>6000000</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" s="13" t="s">
+    <row r="48" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B44">
+      <c r="B48">
         <v>6000000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B45" s="12">
-        <v>1500000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B46">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B47">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="B48">
-        <v>200000</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49">
-        <v>200000</v>
+        <v>54</v>
+      </c>
+      <c r="B49" s="12">
+        <v>1500000</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B50">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B52">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="B50">
+      <c r="B54">
         <v>200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
resolved summing in lease_rent sheet and make parkings dynamic
</commit_message>
<xml_diff>
--- a/artifacts/input.xlsx
+++ b/artifacts/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F9537B-57AA-43CD-886E-58E3AA2E1E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891B226A-CEAF-4B4D-94C9-0B89BA3FD869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Field Name</t>
   </si>
@@ -228,6 +228,12 @@
   </si>
   <si>
     <t>Rate per 2 wheeler</t>
+  </si>
+  <si>
+    <t>Parking Escalation %</t>
+  </si>
+  <si>
+    <t>Parking Escalation Frequency Months</t>
   </si>
 </sst>
 </file>
@@ -358,8 +364,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -694,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79635125-D570-4C1E-9257-DC9C160143A9}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" bestFit="1" customWidth="1"/>
@@ -966,145 +972,145 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="35" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="16" t="s">
+    <row r="35" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="15">
+      <c r="B35">
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="16" t="s">
+    <row r="36" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="15">
+      <c r="B36">
         <v>1500</v>
       </c>
     </row>
-    <row r="37" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="16" t="s">
+    <row r="37" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B37" s="15">
+      <c r="B37">
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:2" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="16" t="s">
+    <row r="38" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B38" s="15">
+      <c r="B38">
         <v>1000</v>
       </c>
     </row>
-    <row r="39" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="B39">
-        <v>110.5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B40">
-        <v>2500000</v>
+    <row r="39" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="15">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="16">
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B41">
-        <v>14000000</v>
+        <v>110.5</v>
       </c>
     </row>
     <row r="42" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B42">
-        <v>5000000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="43" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B43">
-        <v>15000000</v>
+        <v>14000000</v>
       </c>
     </row>
     <row r="44" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B44">
-        <v>14000000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="45" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B45">
-        <v>12000000</v>
+        <v>15000000</v>
       </c>
     </row>
     <row r="46" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B46">
-        <v>5000000</v>
+        <v>14000000</v>
       </c>
     </row>
     <row r="47" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B47">
-        <v>6000000</v>
+        <v>12000000</v>
       </c>
     </row>
     <row r="48" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B48">
-        <v>6000000</v>
+        <v>5000000</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B49" s="12">
-        <v>1500000</v>
+        <v>52</v>
+      </c>
+      <c r="B49">
+        <v>6000000</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B50">
-        <v>200000</v>
+        <v>6000000</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B51">
-        <v>200000</v>
+        <v>54</v>
+      </c>
+      <c r="B51" s="12">
+        <v>1500000</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B52">
         <v>200000</v>
@@ -1112,7 +1118,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B53">
         <v>200000</v>
@@ -1120,9 +1126,25 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B55">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="B54">
+      <c r="B56">
         <v>200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
resolved input merged cell issue
</commit_message>
<xml_diff>
--- a/artifacts/input.xlsx
+++ b/artifacts/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{891B226A-CEAF-4B4D-94C9-0B89BA3FD869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2E3CE2-ED6D-473A-8984-5866AA1B0167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{8983C3BB-AAE5-443A-980D-B8E88AAF0622}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
   <si>
     <t>Field Name</t>
   </si>
@@ -53,9 +53,6 @@
     <t>REU Name</t>
   </si>
   <si>
-    <t>IN-CHEK2</t>
-  </si>
-  <si>
     <t>Lease Type</t>
   </si>
   <si>
@@ -65,15 +62,9 @@
     <t>Building Name</t>
   </si>
   <si>
-    <t>SKCL Tech Park</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
-    <t>Chennai</t>
-  </si>
-  <si>
     <t>Country</t>
   </si>
   <si>
@@ -113,9 +104,6 @@
     <t>Rent Per Sqft</t>
   </si>
   <si>
-    <t>Starting Monthly Rent</t>
-  </si>
-  <si>
     <t>Escalation %</t>
   </si>
   <si>
@@ -134,27 +122,12 @@
     <t>Security Deposit Amount</t>
   </si>
   <si>
-    <t>Refundable Deposit</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Fitout Cost</t>
   </si>
   <si>
     <t>Useful Life Years</t>
   </si>
   <si>
-    <t>Residual Value</t>
-  </si>
-  <si>
-    <t>Discount Rate</t>
-  </si>
-  <si>
-    <t>Incremental Borrowing Rate</t>
-  </si>
-  <si>
     <t>Cost of Capital</t>
   </si>
   <si>
@@ -167,9 +140,6 @@
     <t>Imputed Interest Rate</t>
   </si>
   <si>
-    <t>Ready Reckoner Rate</t>
-  </si>
-  <si>
     <t>Exchange Rate</t>
   </si>
   <si>
@@ -234,13 +204,28 @@
   </si>
   <si>
     <t>Parking Escalation Frequency Months</t>
+  </si>
+  <si>
+    <t>IN-BANN2</t>
+  </si>
+  <si>
+    <t>Nalapad</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>CAM per Sq ft</t>
+  </si>
+  <si>
+    <t>CAM Escalation %</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,11 +264,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
     <font>
       <b/>
@@ -344,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -362,10 +342,9 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79635125-D570-4C1E-9257-DC9C160143A9}">
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" bestFit="1" customWidth="1"/>
@@ -728,106 +707,110 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B9" s="3">
-        <v>9515</v>
+        <v>29750</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B10" s="3">
-        <v>894</v>
+        <f>B9/10.764</f>
+        <v>2763.8424377554816</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B11" s="3">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B12" s="10">
-        <v>46113</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B13" s="10">
-        <v>47938</v>
+        <v>48071</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B14" s="10">
-        <v>46113</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="3"/>
+        <v>19</v>
+      </c>
+      <c r="B15" s="3">
+        <f>(B13-B12)/365*12</f>
+        <v>60</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B16" s="3">
         <v>36</v>
@@ -835,326 +818,299 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B17" s="3">
-        <v>120</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.15</v>
+      </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="4">
-        <v>0.15</v>
+        <v>23</v>
+      </c>
+      <c r="B19" s="13">
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="14">
-        <v>36</v>
+        <v>24</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="B21" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="3">
-        <v>6</v>
+        <v>27</v>
+      </c>
+      <c r="B22" s="5">
+        <v>16869000</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="5">
-        <v>11418000</v>
+        <v>28</v>
+      </c>
+      <c r="B23" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>33</v>
+        <v>59</v>
+      </c>
+      <c r="B24" s="3">
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="3">
-        <v>2000000</v>
+        <v>60</v>
+      </c>
+      <c r="B25" s="15">
+        <v>0.05</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B26" s="3">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="11">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="11">
+        <v>7.1099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="14">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37">
         <v>36</v>
       </c>
-      <c r="B27" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38">
+        <v>110.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="4">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+      <c r="B41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="4">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="B42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="11">
-        <v>0.105</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="7" t="s">
+      <c r="B43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" s="12" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
+      <c r="B44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B32" s="9">
-        <v>500000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" s="13" t="s">
+      <c r="B45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B33" s="11">
-        <v>7.1099999999999997E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="13" t="s">
+      <c r="B46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B34">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B35">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B36">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B37">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B38">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B39" s="15">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" s="16">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="13" t="s">
+      <c r="B47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B41">
-        <v>110.5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="13" t="s">
+      <c r="B48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B42">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="13" t="s">
+      <c r="B49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B43">
-        <v>14000000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="13" t="s">
+      <c r="B50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B44">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="13" t="s">
+      <c r="B51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B45">
-        <v>15000000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="13" t="s">
+      <c r="B52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B46">
-        <v>14000000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47">
-        <v>12000000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49">
-        <v>6000000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B50">
-        <v>6000000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" s="12">
-        <v>1500000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B52">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" s="13" t="s">
-        <v>56</v>
-      </c>
       <c r="B53">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="B54">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56">
-        <v>200000</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="B24" xr:uid="{A4DC2ED1-1DDA-474D-A8CB-950BE676D13B}">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
aligning to the different scenarios
</commit_message>
<xml_diff>
--- a/artifacts/input.xlsx
+++ b/artifacts/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EF1783-2C1F-4B3B-B33A-CE2C63715CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694C0208-6217-4B8C-B9E8-EBE84EE2D0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t>Building Name</t>
   </si>
   <si>
-    <t>Nalapad</t>
-  </si>
-  <si>
     <t>City</t>
   </si>
   <si>
@@ -222,6 +219,9 @@
   </si>
   <si>
     <t>Opex II Per Month</t>
+  </si>
+  <si>
+    <t>Nalapad Bridage</t>
   </si>
 </sst>
 </file>
@@ -283,7 +283,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -317,11 +317,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -342,6 +351,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,53 +730,53 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="3">
-        <v>29750</v>
+        <v>28440</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="3">
         <f>B9/10.764</f>
-        <v>2763.8424377554816</v>
+        <v>2642.1404682274251</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="3">
         <v>0</v>
@@ -774,40 +784,40 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" s="10">
-        <v>46246</v>
+        <v>45947</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" s="10">
-        <v>48071</v>
+        <v>47042</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B14" s="10">
-        <v>46246</v>
+        <v>45947</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="3">
         <f>(B13-B12)/365*12</f>
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="3">
         <v>36</v>
@@ -815,7 +825,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B17" s="3">
         <v>69</v>
@@ -823,7 +833,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B18" s="4">
         <v>0.15</v>
@@ -831,7 +841,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" s="13">
         <v>36</v>
@@ -839,31 +849,31 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="3">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" s="5">
-        <v>16869000</v>
+        <v>18464000</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" s="3">
         <v>0</v>
@@ -871,15 +881,15 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="3">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="15">
         <v>0.05</v>
@@ -887,7 +897,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="3">
         <v>12</v>
@@ -895,15 +905,15 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" s="3">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" s="11">
         <v>0.105</v>
@@ -911,12 +921,15 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="B29" s="16">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30" s="9">
         <v>0</v>
@@ -924,31 +937,31 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B31" s="11">
-        <v>7.1099999999999997E-2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33">
-        <v>4700</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -956,7 +969,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -964,31 +977,31 @@
     </row>
     <row r="36" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B36" s="14">
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B37">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B38">
-        <v>110.5</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -996,15 +1009,15 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B40">
-        <v>5000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -1012,7 +1025,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -1020,7 +1033,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -1028,7 +1041,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -1036,7 +1049,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -1044,7 +1057,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B46">
         <v>0</v>
@@ -1052,7 +1065,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -1060,7 +1073,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -1068,7 +1081,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -1076,7 +1089,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -1084,7 +1097,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -1092,7 +1105,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -1100,7 +1113,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -1108,15 +1121,15 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B54">
-        <v>63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B55">
         <v>0</v>

</xml_diff>